<commit_message>
update second screening A
</commit_message>
<xml_diff>
--- a/lit_review_results/2-screening_phase/second_screening_reviewer_A.xlsx
+++ b/lit_review_results/2-screening_phase/second_screening_reviewer_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wolfrieder/PycharmProjects/sok_artifacts/lit_review_results/2-screening_phase/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFC515FD-570E-A44E-81DA-140FDDC80ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC90EDB4-9EF3-E24F-8D2A-621D56373FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17420" yWindow="-28240" windowWidth="51080" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6603,7 +6603,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -6714,13 +6714,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -6890,8 +6890,6 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -7311,7 +7309,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="2" spans="1:21" s="2" customFormat="1" ht="205" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" s="2" customFormat="1" ht="222" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -7343,7 +7341,7 @@
         <v>1935</v>
       </c>
       <c r="K2" s="60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" s="61" t="b">
         <v>0</v>
@@ -7362,7 +7360,7 @@
         <v>0</v>
       </c>
       <c r="R2" s="72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S2" s="72" t="b">
         <v>0</v>
@@ -7404,7 +7402,7 @@
       </c>
       <c r="J3" s="18"/>
       <c r="K3" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" s="64" t="b">
         <v>0</v>
@@ -7423,7 +7421,7 @@
         <v>0</v>
       </c>
       <c r="R3" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S3" s="75" t="b">
         <v>0</v>
@@ -7465,7 +7463,7 @@
       </c>
       <c r="J4" s="18"/>
       <c r="K4" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4" s="64" t="b">
         <v>0</v>
@@ -7484,7 +7482,7 @@
         <v>0</v>
       </c>
       <c r="R4" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S4" s="75" t="b">
         <v>0</v>
@@ -7528,7 +7526,7 @@
         <v>1716</v>
       </c>
       <c r="K5" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" s="64" t="b">
         <v>0</v>
@@ -7547,7 +7545,7 @@
         <v>0</v>
       </c>
       <c r="R5" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S5" s="75" t="b">
         <v>0</v>
@@ -7591,7 +7589,7 @@
         <v>1930</v>
       </c>
       <c r="K6" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" s="64" t="b">
         <v>0</v>
@@ -7610,7 +7608,7 @@
         <v>0</v>
       </c>
       <c r="R6" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6" s="75" t="b">
         <v>0</v>
@@ -7654,7 +7652,7 @@
         <v>1900</v>
       </c>
       <c r="K7" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" s="64" t="b">
         <v>0</v>
@@ -7673,7 +7671,7 @@
         <v>0</v>
       </c>
       <c r="R7" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" s="75" t="b">
         <v>0</v>
@@ -7717,7 +7715,7 @@
         <v>1855</v>
       </c>
       <c r="K8" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="64" t="b">
         <v>0</v>
@@ -7736,7 +7734,7 @@
         <v>0</v>
       </c>
       <c r="R8" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" s="75" t="b">
         <v>0</v>
@@ -7748,7 +7746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:21" s="4" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" s="4" customFormat="1" ht="155" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
@@ -7780,7 +7778,7 @@
         <v>1820</v>
       </c>
       <c r="K9" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L9" s="64" t="b">
         <v>0</v>
@@ -7799,7 +7797,7 @@
         <v>0</v>
       </c>
       <c r="R9" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9" s="75" t="b">
         <v>0</v>
@@ -7857,7 +7855,7 @@
       </c>
       <c r="P10" s="55"/>
       <c r="Q10" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R10" s="75" t="b">
         <v>0</v>
@@ -7902,7 +7900,7 @@
       </c>
       <c r="J11" s="18"/>
       <c r="K11" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" s="64" t="b">
         <v>0</v>
@@ -7963,19 +7961,19 @@
       </c>
       <c r="J12" s="18"/>
       <c r="K12" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N12" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P12" s="55"/>
       <c r="Q12" s="74" t="b">
@@ -8026,19 +8024,19 @@
         <v>1765</v>
       </c>
       <c r="K13" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N13" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O13" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P13" s="55"/>
       <c r="Q13" s="74" t="b">
@@ -8089,7 +8087,7 @@
         <v>1894</v>
       </c>
       <c r="K14" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" s="64" t="b">
         <v>0</v>
@@ -8108,7 +8106,7 @@
         <v>0</v>
       </c>
       <c r="R14" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" s="75" t="b">
         <v>0</v>
@@ -8152,7 +8150,7 @@
         <v>1797</v>
       </c>
       <c r="K15" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" s="64" t="b">
         <v>0</v>
@@ -8171,7 +8169,7 @@
         <v>0</v>
       </c>
       <c r="R15" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" s="75" t="b">
         <v>0</v>
@@ -8215,7 +8213,7 @@
         <v>1934</v>
       </c>
       <c r="K16" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" s="64" t="b">
         <v>0</v>
@@ -8234,7 +8232,7 @@
         <v>0</v>
       </c>
       <c r="R16" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" s="75" t="b">
         <v>0</v>
@@ -8278,7 +8276,7 @@
         <v>1807</v>
       </c>
       <c r="K17" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" s="64" t="b">
         <v>0</v>
@@ -8297,7 +8295,7 @@
         <v>0</v>
       </c>
       <c r="R17" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" s="75" t="b">
         <v>0</v>
@@ -8341,7 +8339,7 @@
         <v>1737</v>
       </c>
       <c r="K18" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" s="64" t="b">
         <v>0</v>
@@ -8360,7 +8358,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" s="75" t="b">
         <v>0</v>
@@ -8420,7 +8418,7 @@
       </c>
       <c r="P19" s="55"/>
       <c r="Q19" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R19" s="75" t="b">
         <v>0</v>
@@ -8467,7 +8465,7 @@
         <v>1860</v>
       </c>
       <c r="K20" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" s="64" t="b">
         <v>0</v>
@@ -8486,7 +8484,7 @@
         <v>0</v>
       </c>
       <c r="R20" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" s="75" t="b">
         <v>0</v>
@@ -8530,7 +8528,7 @@
         <v>1751</v>
       </c>
       <c r="K21" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="64" t="b">
         <v>0</v>
@@ -8549,7 +8547,7 @@
         <v>0</v>
       </c>
       <c r="R21" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S21" s="75" t="b">
         <v>0</v>
@@ -8593,23 +8591,23 @@
         <v>1845</v>
       </c>
       <c r="K22" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L22" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M22" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P22" s="55"/>
       <c r="Q22" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R22" s="75" t="b">
         <v>0</v>
@@ -8656,19 +8654,19 @@
         <v>1748</v>
       </c>
       <c r="K23" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" s="55"/>
       <c r="Q23" s="74" t="b">
@@ -8719,19 +8717,19 @@
         <v>1741</v>
       </c>
       <c r="K24" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M24" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O24" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P24" s="55"/>
       <c r="Q24" s="74" t="b">
@@ -8782,19 +8780,19 @@
         <v>1843</v>
       </c>
       <c r="K25" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L25" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N25" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P25" s="55"/>
       <c r="Q25" s="74" t="b">
@@ -8845,7 +8843,7 @@
         <v>1811</v>
       </c>
       <c r="K26" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L26" s="64" t="b">
         <v>0</v>
@@ -8864,7 +8862,7 @@
         <v>0</v>
       </c>
       <c r="R26" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S26" s="75" t="b">
         <v>0</v>
@@ -9317,7 +9315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:21" s="4" customFormat="1" ht="155" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" s="4" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>10</v>
       </c>
@@ -9443,7 +9441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:21" s="4" customFormat="1" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" s="4" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>13</v>
       </c>
@@ -10073,7 +10071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:21" s="4" customFormat="1" ht="291" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21" s="4" customFormat="1" ht="274" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>10</v>
       </c>
@@ -10136,7 +10134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:21" s="4" customFormat="1" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21" s="4" customFormat="1" ht="240" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>12</v>
       </c>
@@ -10699,7 +10697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:21" s="4" customFormat="1" ht="358" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" s="4" customFormat="1" ht="325" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>12</v>
       </c>
@@ -10888,7 +10886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:21" s="4" customFormat="1" ht="155" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" s="4" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>12</v>
       </c>
@@ -11262,7 +11260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
         <v>12</v>
       </c>
@@ -11514,7 +11512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:21" s="4" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:21" s="4" customFormat="1" ht="121" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A69" s="32" t="s">
         <v>13</v>
       </c>
@@ -12372,7 +12370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:21" s="4" customFormat="1" ht="155" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:21" s="4" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
         <v>12</v>
       </c>
@@ -13119,7 +13117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:21" s="87" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A95" s="4" t="s">
         <v>13</v>
       </c>
@@ -13165,7 +13163,7 @@
       <c r="O95" s="65" t="b">
         <v>0</v>
       </c>
-      <c r="P95" s="86"/>
+      <c r="P95" s="55"/>
       <c r="Q95" s="74" t="b">
         <v>0</v>
       </c>
@@ -13182,7 +13180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:21" s="4" customFormat="1" ht="325" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:21" s="4" customFormat="1" ht="308" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
         <v>13</v>
       </c>
@@ -13245,7 +13243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A97" s="4" t="s">
         <v>12</v>
       </c>
@@ -15244,7 +15242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:21" s="4" customFormat="1" ht="172" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
         <v>11</v>
       </c>
@@ -15431,7 +15429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:21" s="4" customFormat="1" ht="223" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
         <v>12</v>
       </c>
@@ -16793,7 +16791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:21" s="4" customFormat="1" ht="358" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:21" s="4" customFormat="1" ht="342" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
         <v>12</v>
       </c>
@@ -18614,7 +18612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:21" s="4" customFormat="1" ht="223" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A183" s="4" t="s">
         <v>13</v>
       </c>
@@ -19362,7 +19360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:21" s="4" customFormat="1" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:21" s="4" customFormat="1" ht="240" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A195" s="4" t="s">
         <v>13</v>
       </c>
@@ -19551,7 +19549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A198" s="4" t="s">
         <v>15</v>
       </c>
@@ -20285,7 +20283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:21" s="87" customFormat="1" ht="172" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:21" s="4" customFormat="1" ht="172" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A210" s="4" t="s">
         <v>13</v>
       </c>
@@ -20331,7 +20329,7 @@
       <c r="O210" s="65" t="b">
         <v>0</v>
       </c>
-      <c r="P210" s="86"/>
+      <c r="P210" s="55"/>
       <c r="Q210" s="74" t="b">
         <v>0</v>
       </c>
@@ -20411,7 +20409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:21" s="4" customFormat="1" ht="172" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:21" s="4" customFormat="1" ht="155" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A212" s="4" t="s">
         <v>12</v>
       </c>
@@ -20845,7 +20843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:21" s="4" customFormat="1" ht="358" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:21" s="4" customFormat="1" ht="342" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A219" s="4" t="s">
         <v>14</v>
       </c>
@@ -22260,7 +22258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:21" s="87" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A242" s="4" t="s">
         <v>10</v>
       </c>
@@ -22306,7 +22304,7 @@
       <c r="O242" s="65" t="b">
         <v>0</v>
       </c>
-      <c r="P242" s="86"/>
+      <c r="P242" s="55"/>
       <c r="Q242" s="74" t="b">
         <v>0</v>
       </c>
@@ -22384,7 +22382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:21" s="4" customFormat="1" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:21" s="4" customFormat="1" ht="240" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A244" s="32" t="s">
         <v>13</v>
       </c>
@@ -22488,7 +22486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:21" s="4" customFormat="1" ht="155" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:21" s="4" customFormat="1" ht="172" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A246" s="4" t="s">
         <v>10</v>
       </c>
@@ -23053,7 +23051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:21" s="87" customFormat="1" ht="223" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:21" s="4" customFormat="1" ht="240" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A255" s="4" t="s">
         <v>12</v>
       </c>
@@ -23099,7 +23097,7 @@
       <c r="O255" s="65" t="b">
         <v>0</v>
       </c>
-      <c r="P255" s="86"/>
+      <c r="P255" s="55"/>
       <c r="Q255" s="74" t="b">
         <v>0</v>
       </c>
@@ -23242,7 +23240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:21" s="4" customFormat="1" ht="223" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A258" s="4" t="s">
         <v>13</v>
       </c>
@@ -24998,7 +24996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A286" s="4" t="s">
         <v>13</v>
       </c>
@@ -25876,7 +25874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A300" s="4" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
update second screening xlsx
</commit_message>
<xml_diff>
--- a/lit_review_results/2-screening_phase/second_screening_reviewer_A.xlsx
+++ b/lit_review_results/2-screening_phase/second_screening_reviewer_A.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wolfrieder/PycharmProjects/sok_artifacts/lit_review_results/2-screening_phase/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wolfrieder/Documents/github_repos/sok_artifact_web_tracker_detection/lit_review_results/2-screening_phase/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC90EDB4-9EF3-E24F-8D2A-621D56373FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{428F0FB2-1E92-A149-AEBA-D60029C1A1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17420" yWindow="-28240" windowWidth="51080" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60" yWindow="920" windowWidth="34080" windowHeight="20320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7309,7 +7309,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="2" spans="1:21" s="2" customFormat="1" ht="222" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" s="2" customFormat="1" ht="205" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -7746,7 +7746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:21" s="4" customFormat="1" ht="155" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" s="4" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
@@ -8433,7 +8433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:21" s="4" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" s="4" customFormat="1" ht="121" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>12</v>
       </c>
@@ -8906,7 +8906,7 @@
         <v>1695</v>
       </c>
       <c r="K27" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" s="64" t="b">
         <v>0</v>
@@ -8925,7 +8925,7 @@
         <v>0</v>
       </c>
       <c r="R27" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S27" s="75" t="b">
         <v>0</v>
@@ -8969,7 +8969,7 @@
         <v>1806</v>
       </c>
       <c r="K28" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" s="64" t="b">
         <v>0</v>
@@ -8988,7 +8988,7 @@
         <v>0</v>
       </c>
       <c r="R28" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S28" s="75" t="b">
         <v>0</v>
@@ -9032,7 +9032,7 @@
         <v>1713</v>
       </c>
       <c r="K29" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" s="64" t="b">
         <v>0</v>
@@ -9051,7 +9051,7 @@
         <v>0</v>
       </c>
       <c r="R29" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S29" s="75" t="b">
         <v>0</v>
@@ -9095,7 +9095,7 @@
         <v>1721</v>
       </c>
       <c r="K30" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" s="64" t="b">
         <v>0</v>
@@ -9114,7 +9114,7 @@
         <v>0</v>
       </c>
       <c r="R30" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S30" s="75" t="b">
         <v>0</v>
@@ -9158,19 +9158,19 @@
         <v>1936</v>
       </c>
       <c r="K31" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L31" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M31" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N31" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O31" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P31" s="55"/>
       <c r="Q31" s="74" t="b">
@@ -9221,7 +9221,7 @@
         <v>1699</v>
       </c>
       <c r="K32" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L32" s="64" t="b">
         <v>0</v>
@@ -9240,7 +9240,7 @@
         <v>0</v>
       </c>
       <c r="R32" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S32" s="75" t="b">
         <v>0</v>
@@ -9284,7 +9284,7 @@
         <v>1859</v>
       </c>
       <c r="K33" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" s="64" t="b">
         <v>0</v>
@@ -9303,7 +9303,7 @@
         <v>0</v>
       </c>
       <c r="R33" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S33" s="75" t="b">
         <v>0</v>
@@ -22028,7 +22028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:21" s="4" customFormat="1" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:21" s="4" customFormat="1" ht="240" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A238" s="4" t="s">
         <v>10</v>
       </c>
@@ -22486,7 +22486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:21" s="4" customFormat="1" ht="172" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:21" s="4" customFormat="1" ht="155" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A246" s="4" t="s">
         <v>10</v>
       </c>
@@ -23051,7 +23051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:21" s="4" customFormat="1" ht="240" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:21" s="4" customFormat="1" ht="223" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A255" s="4" t="s">
         <v>12</v>
       </c>
@@ -23240,7 +23240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:21" s="4" customFormat="1" ht="223" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A258" s="4" t="s">
         <v>13</v>
       </c>
@@ -23866,7 +23866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:21" s="4" customFormat="1" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:21" s="4" customFormat="1" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A268" s="4" t="s">
         <v>10</v>
       </c>
@@ -23992,7 +23992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A270" s="4" t="s">
         <v>10</v>
       </c>
@@ -24307,7 +24307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A275" s="4" t="s">
         <v>12</v>
       </c>
@@ -24494,7 +24494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:21" s="4" customFormat="1" ht="240" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:21" s="4" customFormat="1" ht="223" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A278" s="4" t="s">
         <v>15</v>
       </c>
@@ -24996,7 +24996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A286" s="4" t="s">
         <v>13</v>
       </c>
@@ -25874,7 +25874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A300" s="4" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
update second screening A and B
</commit_message>
<xml_diff>
--- a/lit_review_results/2-screening_phase/second_screening_reviewer_A.xlsx
+++ b/lit_review_results/2-screening_phase/second_screening_reviewer_A.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wolfrieder/Documents/github_repos/sok_artifact_web_tracker_detection/lit_review_results/2-screening_phase/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wolfrieder/PycharmProjects/sok_artifacts/lit_review_results/2-screening_phase/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{428F0FB2-1E92-A149-AEBA-D60029C1A1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{311212DC-5D48-C641-84CB-7A784534935D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="920" windowWidth="34080" windowHeight="20320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-7740" yWindow="-28240" windowWidth="51080" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -8433,7 +8433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:21" s="4" customFormat="1" ht="121" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" s="4" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>12</v>
       </c>
@@ -9347,10 +9347,10 @@
         <v>1734</v>
       </c>
       <c r="K34" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L34" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M34" s="64" t="b">
         <v>0</v>
@@ -9369,7 +9369,7 @@
         <v>0</v>
       </c>
       <c r="S34" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T34" s="75" t="b">
         <v>0</v>
@@ -9410,7 +9410,7 @@
         <v>1884</v>
       </c>
       <c r="K35" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35" s="64" t="b">
         <v>0</v>
@@ -9429,7 +9429,7 @@
         <v>0</v>
       </c>
       <c r="R35" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S35" s="75" t="b">
         <v>0</v>
@@ -9473,7 +9473,7 @@
         <v>1889</v>
       </c>
       <c r="K36" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L36" s="64" t="b">
         <v>0</v>
@@ -9492,7 +9492,7 @@
         <v>0</v>
       </c>
       <c r="R36" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S36" s="75" t="b">
         <v>0</v>
@@ -9552,7 +9552,7 @@
       </c>
       <c r="P37" s="55"/>
       <c r="Q37" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R37" s="75" t="b">
         <v>0</v>
@@ -9599,7 +9599,7 @@
         <v>1753</v>
       </c>
       <c r="K38" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" s="64" t="b">
         <v>0</v>
@@ -9618,7 +9618,7 @@
         <v>0</v>
       </c>
       <c r="R38" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S38" s="75" t="b">
         <v>0</v>
@@ -9662,7 +9662,7 @@
         <v>1818</v>
       </c>
       <c r="K39" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" s="64" t="b">
         <v>0</v>
@@ -9681,7 +9681,7 @@
         <v>0</v>
       </c>
       <c r="R39" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S39" s="75" t="b">
         <v>0</v>
@@ -9725,7 +9725,7 @@
         <v>1827</v>
       </c>
       <c r="K40" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L40" s="64" t="b">
         <v>0</v>
@@ -9744,7 +9744,7 @@
         <v>0</v>
       </c>
       <c r="R40" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S40" s="75" t="b">
         <v>0</v>
@@ -9788,7 +9788,7 @@
         <v>1690</v>
       </c>
       <c r="K41" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L41" s="64" t="b">
         <v>0</v>
@@ -9807,7 +9807,7 @@
         <v>0</v>
       </c>
       <c r="R41" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S41" s="75" t="b">
         <v>0</v>
@@ -9851,7 +9851,7 @@
         <v>1749</v>
       </c>
       <c r="K42" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L42" s="64" t="b">
         <v>0</v>
@@ -9870,7 +9870,7 @@
         <v>0</v>
       </c>
       <c r="R42" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S42" s="75" t="b">
         <v>0</v>
@@ -9914,7 +9914,7 @@
         <v>1763</v>
       </c>
       <c r="K43" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" s="64" t="b">
         <v>0</v>
@@ -9933,7 +9933,7 @@
         <v>0</v>
       </c>
       <c r="R43" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S43" s="75" t="b">
         <v>0</v>
@@ -9977,19 +9977,19 @@
         <v>1798</v>
       </c>
       <c r="K44" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L44" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M44" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N44" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O44" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P44" s="55"/>
       <c r="Q44" s="74" t="b">
@@ -10040,19 +10040,19 @@
         <v>1729</v>
       </c>
       <c r="K45" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M45" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N45" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O45" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P45" s="55"/>
       <c r="Q45" s="74" t="b">
@@ -10103,7 +10103,7 @@
         <v>1719</v>
       </c>
       <c r="K46" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L46" s="64" t="b">
         <v>0</v>
@@ -10122,7 +10122,7 @@
         <v>0</v>
       </c>
       <c r="R46" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S46" s="75" t="b">
         <v>0</v>
@@ -10166,7 +10166,7 @@
         <v>1850</v>
       </c>
       <c r="K47" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L47" s="64" t="b">
         <v>0</v>
@@ -10185,7 +10185,7 @@
         <v>0</v>
       </c>
       <c r="R47" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S47" s="75" t="b">
         <v>0</v>
@@ -10229,7 +10229,7 @@
         <v>1865</v>
       </c>
       <c r="K48" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L48" s="64" t="b">
         <v>0</v>
@@ -10248,7 +10248,7 @@
         <v>0</v>
       </c>
       <c r="R48" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S48" s="75" t="b">
         <v>0</v>
@@ -10292,7 +10292,7 @@
         <v>1825</v>
       </c>
       <c r="K49" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" s="64" t="b">
         <v>0</v>
@@ -10311,7 +10311,7 @@
         <v>0</v>
       </c>
       <c r="R49" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S49" s="75" t="b">
         <v>0</v>
@@ -10355,19 +10355,19 @@
         <v>1764</v>
       </c>
       <c r="K50" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L50" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M50" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N50" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O50" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P50" s="55"/>
       <c r="Q50" s="74" t="b">
@@ -10418,19 +10418,19 @@
         <v>1914</v>
       </c>
       <c r="K51" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M51" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N51" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O51" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P51" s="55"/>
       <c r="Q51" s="74" t="b">
@@ -10481,7 +10481,7 @@
         <v>1905</v>
       </c>
       <c r="K52" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L52" s="64" t="b">
         <v>0</v>
@@ -10500,7 +10500,7 @@
         <v>0</v>
       </c>
       <c r="R52" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S52" s="75" t="b">
         <v>0</v>
@@ -10542,7 +10542,7 @@
       </c>
       <c r="J53" s="18"/>
       <c r="K53" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" s="64" t="b">
         <v>0</v>
@@ -10619,7 +10619,7 @@
       </c>
       <c r="P54" s="55"/>
       <c r="Q54" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R54" s="75" t="b">
         <v>0</v>
@@ -10666,7 +10666,7 @@
         <v>1830</v>
       </c>
       <c r="K55" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L55" s="64" t="b">
         <v>0</v>
@@ -10685,7 +10685,7 @@
         <v>0</v>
       </c>
       <c r="R55" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S55" s="75" t="b">
         <v>0</v>
@@ -10745,7 +10745,7 @@
       </c>
       <c r="P56" s="55"/>
       <c r="Q56" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R56" s="75" t="b">
         <v>0</v>
@@ -10792,7 +10792,7 @@
         <v>1762</v>
       </c>
       <c r="K57" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L57" s="64" t="b">
         <v>0</v>
@@ -10811,7 +10811,7 @@
         <v>0</v>
       </c>
       <c r="R57" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S57" s="75" t="b">
         <v>0</v>
@@ -10855,7 +10855,7 @@
         <v>1885</v>
       </c>
       <c r="K58" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L58" s="64" t="b">
         <v>0</v>
@@ -10874,7 +10874,7 @@
         <v>0</v>
       </c>
       <c r="R58" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S58" s="75" t="b">
         <v>0</v>
@@ -10918,7 +10918,7 @@
         <v>1823</v>
       </c>
       <c r="K59" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L59" s="64" t="b">
         <v>0</v>
@@ -10937,7 +10937,7 @@
         <v>0</v>
       </c>
       <c r="R59" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S59" s="75" t="b">
         <v>0</v>
@@ -10979,7 +10979,7 @@
       </c>
       <c r="J60" s="18"/>
       <c r="K60" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L60" s="64" t="b">
         <v>0</v>
@@ -10998,7 +10998,7 @@
         <v>0</v>
       </c>
       <c r="R60" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S60" s="75" t="b">
         <v>0</v>
@@ -11042,10 +11042,10 @@
         <v>1888</v>
       </c>
       <c r="K61" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L61" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M61" s="64" t="b">
         <v>0</v>
@@ -11064,7 +11064,7 @@
         <v>0</v>
       </c>
       <c r="S61" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T61" s="75" t="b">
         <v>0</v>
@@ -11105,7 +11105,7 @@
         <v>1745</v>
       </c>
       <c r="K62" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L62" s="64" t="b">
         <v>0</v>
@@ -11166,7 +11166,7 @@
       </c>
       <c r="J63" s="18"/>
       <c r="K63" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L63" s="64" t="b">
         <v>0</v>
@@ -11185,7 +11185,7 @@
         <v>0</v>
       </c>
       <c r="R63" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S63" s="75" t="b">
         <v>0</v>
@@ -11229,19 +11229,19 @@
         <v>1724</v>
       </c>
       <c r="K64" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L64" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M64" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N64" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O64" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P64" s="55"/>
       <c r="Q64" s="74" t="b">
@@ -11292,7 +11292,7 @@
         <v>1814</v>
       </c>
       <c r="K65" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L65" s="64" t="b">
         <v>0</v>
@@ -11311,7 +11311,7 @@
         <v>0</v>
       </c>
       <c r="R65" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S65" s="75" t="b">
         <v>0</v>
@@ -11355,7 +11355,7 @@
         <v>1916</v>
       </c>
       <c r="K66" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L66" s="64" t="b">
         <v>0</v>
@@ -11374,7 +11374,7 @@
         <v>0</v>
       </c>
       <c r="R66" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S66" s="75" t="b">
         <v>0</v>
@@ -11418,7 +11418,7 @@
         <v>1694</v>
       </c>
       <c r="K67" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L67" s="64" t="b">
         <v>0</v>
@@ -11437,7 +11437,7 @@
         <v>0</v>
       </c>
       <c r="R67" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S67" s="75" t="b">
         <v>0</v>
@@ -11481,19 +11481,19 @@
         <v>1816</v>
       </c>
       <c r="K68" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L68" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M68" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N68" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O68" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P68" s="55"/>
       <c r="Q68" s="74" t="b">
@@ -11587,7 +11587,7 @@
         <v>1732</v>
       </c>
       <c r="K70" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L70" s="64" t="b">
         <v>0</v>
@@ -11606,7 +11606,7 @@
         <v>0</v>
       </c>
       <c r="R70" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S70" s="75" t="b">
         <v>0</v>
@@ -11648,7 +11648,7 @@
       </c>
       <c r="J71" s="18"/>
       <c r="K71" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L71" s="64" t="b">
         <v>0</v>
@@ -11667,7 +11667,7 @@
         <v>0</v>
       </c>
       <c r="R71" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S71" s="75" t="b">
         <v>0</v>
@@ -11711,7 +11711,7 @@
         <v>1784</v>
       </c>
       <c r="K72" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L72" s="64" t="b">
         <v>0</v>
@@ -11730,7 +11730,7 @@
         <v>0</v>
       </c>
       <c r="R72" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S72" s="75" t="b">
         <v>0</v>
@@ -11774,7 +11774,7 @@
         <v>1778</v>
       </c>
       <c r="K73" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L73" s="64" t="b">
         <v>0</v>
@@ -11793,7 +11793,7 @@
         <v>0</v>
       </c>
       <c r="R73" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S73" s="75" t="b">
         <v>0</v>
@@ -11837,7 +11837,7 @@
         <v>1861</v>
       </c>
       <c r="K74" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L74" s="64" t="b">
         <v>0</v>
@@ -11856,7 +11856,7 @@
         <v>0</v>
       </c>
       <c r="R74" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S74" s="75" t="b">
         <v>0</v>
@@ -11900,7 +11900,7 @@
         <v>1740</v>
       </c>
       <c r="K75" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L75" s="64" t="b">
         <v>0</v>
@@ -11919,7 +11919,7 @@
         <v>0</v>
       </c>
       <c r="R75" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S75" s="75" t="b">
         <v>0</v>
@@ -11963,7 +11963,7 @@
         <v>1689</v>
       </c>
       <c r="K76" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L76" s="64" t="b">
         <v>0</v>
@@ -11982,7 +11982,7 @@
         <v>0</v>
       </c>
       <c r="R76" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S76" s="75" t="b">
         <v>0</v>
@@ -12026,7 +12026,7 @@
         <v>1863</v>
       </c>
       <c r="K77" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L77" s="64" t="b">
         <v>0</v>
@@ -12045,7 +12045,7 @@
         <v>0</v>
       </c>
       <c r="R77" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S77" s="75" t="b">
         <v>0</v>
@@ -12089,7 +12089,7 @@
         <v>1836</v>
       </c>
       <c r="K78" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L78" s="64" t="b">
         <v>0</v>
@@ -12108,7 +12108,7 @@
         <v>0</v>
       </c>
       <c r="R78" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S78" s="75" t="b">
         <v>0</v>
@@ -12152,7 +12152,7 @@
         <v>1893</v>
       </c>
       <c r="K79" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L79" s="64" t="b">
         <v>0</v>
@@ -12171,7 +12171,7 @@
         <v>0</v>
       </c>
       <c r="R79" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S79" s="75" t="b">
         <v>0</v>
@@ -12215,16 +12215,16 @@
         <v>1817</v>
       </c>
       <c r="K80" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L80" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M80" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N80" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O80" s="65" t="b">
         <v>0</v>
@@ -12276,7 +12276,7 @@
       </c>
       <c r="J81" s="18"/>
       <c r="K81" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L81" s="64" t="b">
         <v>0</v>
@@ -12295,7 +12295,7 @@
         <v>0</v>
       </c>
       <c r="R81" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S81" s="75" t="b">
         <v>0</v>
@@ -12339,7 +12339,7 @@
         <v>1929</v>
       </c>
       <c r="K82" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" s="64" t="b">
         <v>0</v>
@@ -12358,7 +12358,7 @@
         <v>0</v>
       </c>
       <c r="R82" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S82" s="75" t="b">
         <v>0</v>
@@ -12402,7 +12402,7 @@
         <v>1839</v>
       </c>
       <c r="K83" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L83" s="64" t="b">
         <v>0</v>
@@ -12421,7 +12421,7 @@
         <v>0</v>
       </c>
       <c r="R83" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S83" s="75" t="b">
         <v>0</v>
@@ -12465,7 +12465,7 @@
         <v>1838</v>
       </c>
       <c r="K84" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L84" s="64" t="b">
         <v>0</v>
@@ -12484,7 +12484,7 @@
         <v>0</v>
       </c>
       <c r="R84" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S84" s="75" t="b">
         <v>0</v>
@@ -12526,7 +12526,7 @@
       </c>
       <c r="J85" s="18"/>
       <c r="K85" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L85" s="64" t="b">
         <v>0</v>
@@ -12545,7 +12545,7 @@
         <v>0</v>
       </c>
       <c r="R85" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S85" s="75" t="b">
         <v>0</v>
@@ -12589,19 +12589,19 @@
         <v>1857</v>
       </c>
       <c r="K86" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L86" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M86" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N86" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O86" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P86" s="55"/>
       <c r="Q86" s="74" t="b">
@@ -12652,19 +12652,19 @@
         <v>1775</v>
       </c>
       <c r="K87" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L87" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M87" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N87" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O87" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P87" s="55"/>
       <c r="Q87" s="74" t="b">
@@ -12715,7 +12715,7 @@
         <v>1890</v>
       </c>
       <c r="K88" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L88" s="64" t="b">
         <v>0</v>
@@ -12734,7 +12734,7 @@
         <v>0</v>
       </c>
       <c r="R88" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S88" s="75" t="b">
         <v>0</v>
@@ -12778,7 +12778,7 @@
         <v>1738</v>
       </c>
       <c r="K89" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L89" s="64" t="b">
         <v>0</v>
@@ -12797,7 +12797,7 @@
         <v>0</v>
       </c>
       <c r="R89" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S89" s="75" t="b">
         <v>0</v>
@@ -12841,7 +12841,7 @@
         <v>1707</v>
       </c>
       <c r="K90" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L90" s="64" t="b">
         <v>0</v>
@@ -12860,7 +12860,7 @@
         <v>0</v>
       </c>
       <c r="R90" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S90" s="75" t="b">
         <v>0</v>
@@ -12904,7 +12904,7 @@
         <v>1708</v>
       </c>
       <c r="K91" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L91" s="64" t="b">
         <v>0</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="R91" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S91" s="75" t="b">
         <v>0</v>
@@ -12967,7 +12967,7 @@
         <v>1833</v>
       </c>
       <c r="K92" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L92" s="64" t="b">
         <v>0</v>
@@ -12986,7 +12986,7 @@
         <v>0</v>
       </c>
       <c r="R92" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S92" s="75" t="b">
         <v>0</v>
@@ -13046,7 +13046,7 @@
       </c>
       <c r="P93" s="55"/>
       <c r="Q93" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R93" s="75" t="b">
         <v>0</v>
@@ -13086,19 +13086,19 @@
       </c>
       <c r="J94" s="18"/>
       <c r="K94" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L94" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M94" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N94" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O94" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P94" s="55"/>
       <c r="Q94" s="74" t="b">
@@ -13149,19 +13149,19 @@
         <v>1876</v>
       </c>
       <c r="K95" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L95" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M95" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N95" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O95" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P95" s="55"/>
       <c r="Q95" s="74" t="b">
@@ -13212,7 +13212,7 @@
         <v>1869</v>
       </c>
       <c r="K96" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L96" s="64" t="b">
         <v>0</v>
@@ -13231,7 +13231,7 @@
         <v>0</v>
       </c>
       <c r="R96" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S96" s="75" t="b">
         <v>0</v>
@@ -13275,7 +13275,7 @@
         <v>1812</v>
       </c>
       <c r="K97" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L97" s="64" t="b">
         <v>0</v>
@@ -13294,7 +13294,7 @@
         <v>0</v>
       </c>
       <c r="R97" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S97" s="75" t="b">
         <v>0</v>
@@ -13338,7 +13338,7 @@
         <v>1901</v>
       </c>
       <c r="K98" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L98" s="64" t="b">
         <v>0</v>
@@ -13357,7 +13357,7 @@
         <v>0</v>
       </c>
       <c r="R98" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S98" s="75" t="b">
         <v>0</v>
@@ -13401,7 +13401,7 @@
         <v>1799</v>
       </c>
       <c r="K99" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L99" s="64" t="b">
         <v>0</v>
@@ -13420,7 +13420,7 @@
         <v>0</v>
       </c>
       <c r="R99" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S99" s="75" t="b">
         <v>0</v>
@@ -13464,7 +13464,7 @@
         <v>1804</v>
       </c>
       <c r="K100" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L100" s="64" t="b">
         <v>0</v>
@@ -13483,7 +13483,7 @@
         <v>0</v>
       </c>
       <c r="R100" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S100" s="75" t="b">
         <v>0</v>
@@ -13527,7 +13527,7 @@
         <v>1736</v>
       </c>
       <c r="K101" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L101" s="64" t="b">
         <v>0</v>
@@ -13546,7 +13546,7 @@
         <v>0</v>
       </c>
       <c r="R101" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S101" s="75" t="b">
         <v>0</v>
@@ -13590,10 +13590,10 @@
         <v>1864</v>
       </c>
       <c r="K102" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L102" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M102" s="64" t="b">
         <v>0</v>
@@ -13612,7 +13612,7 @@
         <v>0</v>
       </c>
       <c r="S102" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T102" s="75" t="b">
         <v>0</v>
@@ -13653,7 +13653,7 @@
         <v>1851</v>
       </c>
       <c r="K103" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L103" s="64" t="b">
         <v>0</v>
@@ -13672,7 +13672,7 @@
         <v>0</v>
       </c>
       <c r="R103" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S103" s="75" t="b">
         <v>0</v>
@@ -13716,7 +13716,7 @@
         <v>1711</v>
       </c>
       <c r="K104" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L104" s="64" t="b">
         <v>0</v>
@@ -13735,7 +13735,7 @@
         <v>0</v>
       </c>
       <c r="R104" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S104" s="75" t="b">
         <v>0</v>
@@ -13779,7 +13779,7 @@
         <v>1920</v>
       </c>
       <c r="K105" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L105" s="64" t="b">
         <v>0</v>
@@ -13798,7 +13798,7 @@
         <v>0</v>
       </c>
       <c r="R105" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S105" s="75" t="b">
         <v>0</v>
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J106" s="18"/>
       <c r="K106" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L106" s="64" t="b">
         <v>0</v>
@@ -13859,7 +13859,7 @@
         <v>0</v>
       </c>
       <c r="R106" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S106" s="75" t="b">
         <v>0</v>
@@ -13901,7 +13901,7 @@
       </c>
       <c r="J107" s="18"/>
       <c r="K107" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L107" s="64" t="b">
         <v>0</v>
@@ -13920,7 +13920,7 @@
         <v>0</v>
       </c>
       <c r="R107" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S107" s="75" t="b">
         <v>0</v>
@@ -13964,7 +13964,7 @@
         <v>1903</v>
       </c>
       <c r="K108" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L108" s="64" t="b">
         <v>0</v>
@@ -13983,7 +13983,7 @@
         <v>0</v>
       </c>
       <c r="R108" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S108" s="75" t="b">
         <v>0</v>
@@ -14027,7 +14027,7 @@
         <v>1910</v>
       </c>
       <c r="K109" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L109" s="64" t="b">
         <v>0</v>
@@ -14046,7 +14046,7 @@
         <v>0</v>
       </c>
       <c r="R109" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S109" s="75" t="b">
         <v>0</v>
@@ -14088,7 +14088,7 @@
       </c>
       <c r="J110" s="18"/>
       <c r="K110" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L110" s="64" t="b">
         <v>0</v>
@@ -14107,7 +14107,7 @@
         <v>0</v>
       </c>
       <c r="R110" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S110" s="75" t="b">
         <v>0</v>
@@ -14151,7 +14151,7 @@
         <v>1891</v>
       </c>
       <c r="K111" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L111" s="64" t="b">
         <v>0</v>
@@ -14170,7 +14170,7 @@
         <v>0</v>
       </c>
       <c r="R111" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S111" s="75" t="b">
         <v>0</v>
@@ -14214,7 +14214,7 @@
         <v>1696</v>
       </c>
       <c r="K112" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L112" s="64" t="b">
         <v>0</v>
@@ -14233,7 +14233,7 @@
         <v>0</v>
       </c>
       <c r="R112" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S112" s="75" t="b">
         <v>0</v>
@@ -14277,7 +14277,7 @@
         <v>1896</v>
       </c>
       <c r="K113" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L113" s="64" t="b">
         <v>0</v>
@@ -14296,7 +14296,7 @@
         <v>0</v>
       </c>
       <c r="R113" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S113" s="75" t="b">
         <v>0</v>
@@ -14338,7 +14338,7 @@
       </c>
       <c r="J114" s="18"/>
       <c r="K114" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L114" s="64" t="b">
         <v>0</v>
@@ -14357,7 +14357,7 @@
         <v>0</v>
       </c>
       <c r="R114" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S114" s="75" t="b">
         <v>0</v>
@@ -14401,7 +14401,7 @@
         <v>1735</v>
       </c>
       <c r="K115" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L115" s="64" t="b">
         <v>0</v>
@@ -14420,7 +14420,7 @@
         <v>0</v>
       </c>
       <c r="R115" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S115" s="75" t="b">
         <v>0</v>
@@ -14464,7 +14464,7 @@
         <v>1767</v>
       </c>
       <c r="K116" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L116" s="64" t="b">
         <v>0</v>
@@ -14483,7 +14483,7 @@
         <v>0</v>
       </c>
       <c r="R116" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S116" s="75" t="b">
         <v>0</v>
@@ -14527,7 +14527,7 @@
         <v>1750</v>
       </c>
       <c r="K117" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L117" s="64" t="b">
         <v>0</v>
@@ -14546,7 +14546,7 @@
         <v>0</v>
       </c>
       <c r="R117" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S117" s="75" t="b">
         <v>0</v>
@@ -14590,19 +14590,19 @@
         <v>1844</v>
       </c>
       <c r="K118" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L118" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M118" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N118" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O118" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P118" s="55"/>
       <c r="Q118" s="74" t="b">
@@ -14653,7 +14653,7 @@
         <v>1768</v>
       </c>
       <c r="K119" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L119" s="64" t="b">
         <v>0</v>
@@ -14672,7 +14672,7 @@
         <v>0</v>
       </c>
       <c r="R119" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S119" s="75" t="b">
         <v>0</v>
@@ -14716,7 +14716,7 @@
         <v>1858</v>
       </c>
       <c r="K120" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L120" s="64" t="b">
         <v>0</v>
@@ -14735,7 +14735,7 @@
         <v>0</v>
       </c>
       <c r="R120" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S120" s="75" t="b">
         <v>0</v>
@@ -14779,7 +14779,7 @@
         <v>1693</v>
       </c>
       <c r="K121" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L121" s="64" t="b">
         <v>0</v>
@@ -14798,7 +14798,7 @@
         <v>0</v>
       </c>
       <c r="R121" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S121" s="75" t="b">
         <v>0</v>
@@ -14842,7 +14842,7 @@
         <v>1846</v>
       </c>
       <c r="K122" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L122" s="64" t="b">
         <v>0</v>
@@ -14861,7 +14861,7 @@
         <v>0</v>
       </c>
       <c r="R122" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S122" s="75" t="b">
         <v>0</v>
@@ -14905,7 +14905,7 @@
         <v>1754</v>
       </c>
       <c r="K123" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L123" s="64" t="b">
         <v>0</v>
@@ -14924,7 +14924,7 @@
         <v>0</v>
       </c>
       <c r="R123" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S123" s="75" t="b">
         <v>0</v>
@@ -14977,7 +14977,7 @@
       </c>
       <c r="P124" s="55"/>
       <c r="Q124" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R124" s="75" t="b">
         <v>0</v>
@@ -15024,19 +15024,19 @@
         <v>1927</v>
       </c>
       <c r="K125" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L125" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M125" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N125" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O125" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P125" s="55"/>
       <c r="Q125" s="74" t="b">
@@ -15085,7 +15085,7 @@
       </c>
       <c r="J126" s="18"/>
       <c r="K126" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L126" s="64" t="b">
         <v>0</v>
@@ -15104,7 +15104,7 @@
         <v>0</v>
       </c>
       <c r="R126" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S126" s="75" t="b">
         <v>0</v>
@@ -15148,7 +15148,7 @@
         <v>1862</v>
       </c>
       <c r="K127" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L127" s="64" t="b">
         <v>0</v>
@@ -15167,7 +15167,7 @@
         <v>0</v>
       </c>
       <c r="R127" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S127" s="75" t="b">
         <v>0</v>
@@ -15211,19 +15211,19 @@
         <v>1917</v>
       </c>
       <c r="K128" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L128" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M128" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N128" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O128" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P128" s="55"/>
       <c r="Q128" s="74" t="b">
@@ -15274,19 +15274,19 @@
         <v>1757</v>
       </c>
       <c r="K129" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L129" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M129" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N129" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O129" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P129" s="55"/>
       <c r="Q129" s="74" t="b">
@@ -15337,19 +15337,19 @@
         <v>1760</v>
       </c>
       <c r="K130" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L130" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M130" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N130" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O130" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P130" s="55"/>
       <c r="Q130" s="74" t="b">
@@ -15398,7 +15398,7 @@
       </c>
       <c r="J131" s="18"/>
       <c r="K131" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L131" s="64" t="b">
         <v>0</v>
@@ -15417,7 +15417,7 @@
         <v>0</v>
       </c>
       <c r="R131" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S131" s="75" t="b">
         <v>0</v>
@@ -15461,10 +15461,10 @@
         <v>1840</v>
       </c>
       <c r="K132" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L132" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M132" s="64" t="b">
         <v>0</v>
@@ -15483,7 +15483,7 @@
         <v>0</v>
       </c>
       <c r="S132" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T132" s="75" t="b">
         <v>0</v>
@@ -15522,7 +15522,7 @@
       </c>
       <c r="J133" s="18"/>
       <c r="K133" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L133" s="64" t="b">
         <v>0</v>
@@ -15541,7 +15541,7 @@
         <v>0</v>
       </c>
       <c r="R133" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S133" s="75" t="b">
         <v>0</v>
@@ -15580,7 +15580,7 @@
       </c>
       <c r="J134" s="18"/>
       <c r="K134" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L134" s="64" t="b">
         <v>0</v>
@@ -15599,7 +15599,7 @@
         <v>0</v>
       </c>
       <c r="R134" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S134" s="75" t="b">
         <v>0</v>
@@ -15643,7 +15643,7 @@
         <v>1743</v>
       </c>
       <c r="K135" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L135" s="64" t="b">
         <v>0</v>
@@ -15662,7 +15662,7 @@
         <v>0</v>
       </c>
       <c r="R135" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S135" s="75" t="b">
         <v>0</v>
@@ -15706,7 +15706,7 @@
         <v>1788</v>
       </c>
       <c r="K136" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L136" s="64" t="b">
         <v>0</v>
@@ -15725,7 +15725,7 @@
         <v>0</v>
       </c>
       <c r="R136" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S136" s="75" t="b">
         <v>0</v>
@@ -15785,7 +15785,7 @@
       </c>
       <c r="P137" s="55"/>
       <c r="Q137" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R137" s="75" t="b">
         <v>0</v>
@@ -15832,7 +15832,7 @@
         <v>1691</v>
       </c>
       <c r="K138" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L138" s="64" t="b">
         <v>0</v>
@@ -15851,7 +15851,7 @@
         <v>0</v>
       </c>
       <c r="R138" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S138" s="75" t="b">
         <v>0</v>
@@ -15891,7 +15891,7 @@
       </c>
       <c r="J139" s="18"/>
       <c r="K139" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L139" s="64" t="b">
         <v>0</v>
@@ -15910,7 +15910,7 @@
         <v>0</v>
       </c>
       <c r="R139" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S139" s="75" t="b">
         <v>0</v>
@@ -15954,7 +15954,7 @@
         <v>1878</v>
       </c>
       <c r="K140" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L140" s="64" t="b">
         <v>0</v>
@@ -15973,7 +15973,7 @@
         <v>0</v>
       </c>
       <c r="R140" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S140" s="75" t="b">
         <v>0</v>
@@ -16015,7 +16015,7 @@
       </c>
       <c r="J141" s="18"/>
       <c r="K141" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L141" s="64" t="b">
         <v>0</v>
@@ -16034,7 +16034,7 @@
         <v>0</v>
       </c>
       <c r="R141" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S141" s="75" t="b">
         <v>0</v>
@@ -16078,7 +16078,7 @@
         <v>1913</v>
       </c>
       <c r="K142" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L142" s="64" t="b">
         <v>0</v>
@@ -16097,7 +16097,7 @@
         <v>0</v>
       </c>
       <c r="R142" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S142" s="75" t="b">
         <v>0</v>
@@ -16157,7 +16157,7 @@
       </c>
       <c r="P143" s="55"/>
       <c r="Q143" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R143" s="75" t="b">
         <v>0</v>
@@ -16204,7 +16204,7 @@
         <v>1899</v>
       </c>
       <c r="K144" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L144" s="64" t="b">
         <v>0</v>
@@ -16223,7 +16223,7 @@
         <v>0</v>
       </c>
       <c r="R144" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S144" s="75" t="b">
         <v>0</v>
@@ -16267,7 +16267,7 @@
         <v>1803</v>
       </c>
       <c r="K145" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L145" s="64" t="b">
         <v>0</v>
@@ -16286,7 +16286,7 @@
         <v>0</v>
       </c>
       <c r="R145" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S145" s="75" t="b">
         <v>0</v>
@@ -16330,7 +16330,7 @@
         <v>1832</v>
       </c>
       <c r="K146" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L146" s="64" t="b">
         <v>0</v>
@@ -16349,7 +16349,7 @@
         <v>0</v>
       </c>
       <c r="R146" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S146" s="75" t="b">
         <v>0</v>
@@ -16386,7 +16386,7 @@
       </c>
       <c r="J147" s="18"/>
       <c r="K147" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L147" s="64" t="b">
         <v>0</v>
@@ -16405,7 +16405,7 @@
         <v>0</v>
       </c>
       <c r="R147" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S147" s="75" t="b">
         <v>0</v>
@@ -16463,7 +16463,7 @@
       </c>
       <c r="P148" s="55"/>
       <c r="Q148" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R148" s="75" t="b">
         <v>0</v>
@@ -16510,7 +16510,7 @@
         <v>1723</v>
       </c>
       <c r="K149" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L149" s="64" t="b">
         <v>0</v>
@@ -16529,7 +16529,7 @@
         <v>0</v>
       </c>
       <c r="R149" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S149" s="75" t="b">
         <v>0</v>
@@ -16573,7 +16573,7 @@
         <v>1933</v>
       </c>
       <c r="K150" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L150" s="64" t="b">
         <v>0</v>
@@ -16592,7 +16592,7 @@
         <v>0</v>
       </c>
       <c r="R150" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S150" s="75" t="b">
         <v>0</v>
@@ -16634,7 +16634,7 @@
       </c>
       <c r="J151" s="18"/>
       <c r="K151" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L151" s="64" t="b">
         <v>0</v>
@@ -16653,7 +16653,7 @@
         <v>0</v>
       </c>
       <c r="R151" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S151" s="75" t="b">
         <v>0</v>
@@ -16697,7 +16697,7 @@
         <v>1870</v>
       </c>
       <c r="K152" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L152" s="64" t="b">
         <v>0</v>
@@ -16716,7 +16716,7 @@
         <v>0</v>
       </c>
       <c r="R152" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S152" s="75" t="b">
         <v>0</v>
@@ -16760,7 +16760,7 @@
         <v>1912</v>
       </c>
       <c r="K153" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L153" s="64" t="b">
         <v>0</v>
@@ -16779,7 +16779,7 @@
         <v>0</v>
       </c>
       <c r="R153" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S153" s="75" t="b">
         <v>0</v>
@@ -16823,7 +16823,7 @@
         <v>1831</v>
       </c>
       <c r="K154" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L154" s="64" t="b">
         <v>0</v>
@@ -16842,7 +16842,7 @@
         <v>0</v>
       </c>
       <c r="R154" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S154" s="75" t="b">
         <v>0</v>
@@ -16884,7 +16884,7 @@
       </c>
       <c r="J155" s="18"/>
       <c r="K155" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L155" s="64" t="b">
         <v>0</v>
@@ -16903,7 +16903,7 @@
         <v>0</v>
       </c>
       <c r="R155" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S155" s="75" t="b">
         <v>0</v>
@@ -16947,7 +16947,7 @@
         <v>1872</v>
       </c>
       <c r="K156" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L156" s="64" t="b">
         <v>0</v>
@@ -16966,7 +16966,7 @@
         <v>0</v>
       </c>
       <c r="R156" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S156" s="75" t="b">
         <v>0</v>
@@ -17010,19 +17010,19 @@
         <v>1874</v>
       </c>
       <c r="K157" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L157" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M157" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N157" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O157" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P157" s="55"/>
       <c r="Q157" s="74" t="b">
@@ -17073,19 +17073,19 @@
         <v>1761</v>
       </c>
       <c r="K158" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L158" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M158" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N158" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O158" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P158" s="55"/>
       <c r="Q158" s="74" t="b">
@@ -17136,7 +17136,7 @@
         <v>1705</v>
       </c>
       <c r="K159" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L159" s="64" t="b">
         <v>0</v>
@@ -17155,7 +17155,7 @@
         <v>0</v>
       </c>
       <c r="R159" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S159" s="75" t="b">
         <v>0</v>
@@ -17199,19 +17199,19 @@
         <v>1774</v>
       </c>
       <c r="K160" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L160" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M160" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N160" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O160" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P160" s="55"/>
       <c r="Q160" s="74" t="b">
@@ -17262,7 +17262,7 @@
         <v>1932</v>
       </c>
       <c r="K161" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L161" s="64" t="b">
         <v>0</v>
@@ -17281,7 +17281,7 @@
         <v>0</v>
       </c>
       <c r="R161" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S161" s="75" t="b">
         <v>0</v>
@@ -17325,7 +17325,7 @@
         <v>1781</v>
       </c>
       <c r="K162" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L162" s="64" t="b">
         <v>0</v>
@@ -17344,7 +17344,7 @@
         <v>0</v>
       </c>
       <c r="R162" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S162" s="75" t="b">
         <v>0</v>
@@ -17388,7 +17388,7 @@
         <v>1722</v>
       </c>
       <c r="K163" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L163" s="64" t="b">
         <v>0</v>
@@ -17407,7 +17407,7 @@
         <v>0</v>
       </c>
       <c r="R163" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S163" s="75" t="b">
         <v>0</v>
@@ -17451,7 +17451,7 @@
         <v>1842</v>
       </c>
       <c r="K164" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L164" s="64" t="b">
         <v>0</v>
@@ -17470,7 +17470,7 @@
         <v>0</v>
       </c>
       <c r="R164" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S164" s="75" t="b">
         <v>0</v>
@@ -17514,7 +17514,7 @@
         <v>1810</v>
       </c>
       <c r="K165" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L165" s="64" t="b">
         <v>0</v>
@@ -17533,7 +17533,7 @@
         <v>0</v>
       </c>
       <c r="R165" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S165" s="75" t="b">
         <v>0</v>
@@ -17577,7 +17577,7 @@
         <v>1931</v>
       </c>
       <c r="K166" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L166" s="64" t="b">
         <v>0</v>
@@ -17596,7 +17596,7 @@
         <v>0</v>
       </c>
       <c r="R166" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S166" s="75" t="b">
         <v>0</v>
@@ -17640,7 +17640,7 @@
         <v>1837</v>
       </c>
       <c r="K167" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L167" s="64" t="b">
         <v>0</v>
@@ -17659,7 +17659,7 @@
         <v>0</v>
       </c>
       <c r="R167" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S167" s="75" t="b">
         <v>0</v>
@@ -17703,7 +17703,7 @@
         <v>1928</v>
       </c>
       <c r="K168" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L168" s="64" t="b">
         <v>0</v>
@@ -17722,7 +17722,7 @@
         <v>0</v>
       </c>
       <c r="R168" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S168" s="75" t="b">
         <v>0</v>
@@ -17766,7 +17766,7 @@
         <v>1704</v>
       </c>
       <c r="K169" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L169" s="64" t="b">
         <v>0</v>
@@ -17785,7 +17785,7 @@
         <v>0</v>
       </c>
       <c r="R169" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S169" s="75" t="b">
         <v>0</v>
@@ -17829,7 +17829,7 @@
         <v>1759</v>
       </c>
       <c r="K170" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L170" s="64" t="b">
         <v>0</v>
@@ -17848,7 +17848,7 @@
         <v>0</v>
       </c>
       <c r="R170" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S170" s="75" t="b">
         <v>0</v>
@@ -17892,7 +17892,7 @@
         <v>1881</v>
       </c>
       <c r="K171" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L171" s="64" t="b">
         <v>0</v>
@@ -17911,7 +17911,7 @@
         <v>0</v>
       </c>
       <c r="R171" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S171" s="75" t="b">
         <v>0</v>
@@ -17955,19 +17955,19 @@
         <v>1739</v>
       </c>
       <c r="K172" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L172" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M172" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N172" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O172" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P172" s="55"/>
       <c r="Q172" s="74" t="b">
@@ -18018,7 +18018,7 @@
         <v>1854</v>
       </c>
       <c r="K173" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L173" s="64" t="b">
         <v>0</v>
@@ -18037,7 +18037,7 @@
         <v>0</v>
       </c>
       <c r="R173" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S173" s="75" t="b">
         <v>0</v>
@@ -18081,7 +18081,7 @@
         <v>1925</v>
       </c>
       <c r="K174" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L174" s="64" t="b">
         <v>0</v>
@@ -18100,7 +18100,7 @@
         <v>0</v>
       </c>
       <c r="R174" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S174" s="75" t="b">
         <v>0</v>
@@ -18144,7 +18144,7 @@
         <v>1720</v>
       </c>
       <c r="K175" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L175" s="64" t="b">
         <v>0</v>
@@ -18163,7 +18163,7 @@
         <v>0</v>
       </c>
       <c r="R175" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S175" s="75" t="b">
         <v>0</v>
@@ -18205,7 +18205,7 @@
       </c>
       <c r="J176" s="18"/>
       <c r="K176" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L176" s="64" t="b">
         <v>0</v>
@@ -18224,7 +18224,7 @@
         <v>0</v>
       </c>
       <c r="R176" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S176" s="75" t="b">
         <v>0</v>
@@ -18268,7 +18268,7 @@
         <v>1815</v>
       </c>
       <c r="K177" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L177" s="64" t="b">
         <v>0</v>
@@ -18287,7 +18287,7 @@
         <v>0</v>
       </c>
       <c r="R177" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S177" s="75" t="b">
         <v>0</v>
@@ -18331,7 +18331,7 @@
         <v>1726</v>
       </c>
       <c r="K178" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L178" s="64" t="b">
         <v>0</v>
@@ -18350,7 +18350,7 @@
         <v>0</v>
       </c>
       <c r="R178" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S178" s="75" t="b">
         <v>0</v>
@@ -18394,7 +18394,7 @@
         <v>1725</v>
       </c>
       <c r="K179" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L179" s="64" t="b">
         <v>0</v>
@@ -18413,7 +18413,7 @@
         <v>0</v>
       </c>
       <c r="R179" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S179" s="75" t="b">
         <v>0</v>
@@ -18457,7 +18457,7 @@
         <v>1923</v>
       </c>
       <c r="K180" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L180" s="64" t="b">
         <v>0</v>
@@ -18476,7 +18476,7 @@
         <v>0</v>
       </c>
       <c r="R180" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S180" s="75" t="b">
         <v>0</v>
@@ -18520,7 +18520,7 @@
         <v>1907</v>
       </c>
       <c r="K181" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L181" s="64" t="b">
         <v>0</v>
@@ -18539,7 +18539,7 @@
         <v>0</v>
       </c>
       <c r="R181" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S181" s="75" t="b">
         <v>0</v>
@@ -18581,7 +18581,7 @@
       </c>
       <c r="J182" s="18"/>
       <c r="K182" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L182" s="64" t="b">
         <v>0</v>
@@ -18600,7 +18600,7 @@
         <v>0</v>
       </c>
       <c r="R182" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S182" s="75" t="b">
         <v>0</v>
@@ -18644,7 +18644,7 @@
         <v>1892</v>
       </c>
       <c r="K183" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L183" s="64" t="b">
         <v>0</v>
@@ -18663,7 +18663,7 @@
         <v>0</v>
       </c>
       <c r="R183" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S183" s="75" t="b">
         <v>0</v>
@@ -18707,7 +18707,7 @@
         <v>1902</v>
       </c>
       <c r="K184" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L184" s="64" t="b">
         <v>0</v>
@@ -18726,7 +18726,7 @@
         <v>0</v>
       </c>
       <c r="R184" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S184" s="75" t="b">
         <v>0</v>
@@ -18770,7 +18770,7 @@
         <v>1687</v>
       </c>
       <c r="K185" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L185" s="64" t="b">
         <v>0</v>
@@ -18789,7 +18789,7 @@
         <v>0</v>
       </c>
       <c r="R185" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S185" s="75" t="b">
         <v>0</v>
@@ -18833,7 +18833,7 @@
         <v>1866</v>
       </c>
       <c r="K186" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L186" s="64" t="b">
         <v>0</v>
@@ -18852,7 +18852,7 @@
         <v>0</v>
       </c>
       <c r="R186" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S186" s="75" t="b">
         <v>0</v>
@@ -18896,7 +18896,7 @@
         <v>1886</v>
       </c>
       <c r="K187" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L187" s="64" t="b">
         <v>0</v>
@@ -18915,7 +18915,7 @@
         <v>0</v>
       </c>
       <c r="R187" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S187" s="75" t="b">
         <v>0</v>
@@ -18957,7 +18957,7 @@
       </c>
       <c r="J188" s="18"/>
       <c r="K188" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L188" s="64" t="b">
         <v>0</v>
@@ -18976,7 +18976,7 @@
         <v>0</v>
       </c>
       <c r="R188" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S188" s="75" t="b">
         <v>0</v>
@@ -19020,7 +19020,7 @@
         <v>1849</v>
       </c>
       <c r="K189" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L189" s="64" t="b">
         <v>0</v>
@@ -19039,7 +19039,7 @@
         <v>0</v>
       </c>
       <c r="R189" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S189" s="75" t="b">
         <v>0</v>
@@ -19079,7 +19079,7 @@
       </c>
       <c r="J190" s="18"/>
       <c r="K190" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L190" s="64" t="b">
         <v>0</v>
@@ -19098,7 +19098,7 @@
         <v>0</v>
       </c>
       <c r="R190" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S190" s="75" t="b">
         <v>0</v>
@@ -19140,7 +19140,7 @@
       </c>
       <c r="J191" s="18"/>
       <c r="K191" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L191" s="64" t="b">
         <v>0</v>
@@ -19159,7 +19159,7 @@
         <v>0</v>
       </c>
       <c r="R191" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S191" s="75" t="b">
         <v>0</v>
@@ -19203,7 +19203,7 @@
         <v>1791</v>
       </c>
       <c r="K192" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L192" s="64" t="b">
         <v>0</v>
@@ -19222,7 +19222,7 @@
         <v>0</v>
       </c>
       <c r="R192" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S192" s="75" t="b">
         <v>0</v>
@@ -19266,7 +19266,7 @@
         <v>1904</v>
       </c>
       <c r="K193" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L193" s="64" t="b">
         <v>0</v>
@@ -19285,7 +19285,7 @@
         <v>0</v>
       </c>
       <c r="R193" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S193" s="75" t="b">
         <v>0</v>
@@ -19329,7 +19329,7 @@
         <v>1727</v>
       </c>
       <c r="K194" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L194" s="64" t="b">
         <v>0</v>
@@ -19348,7 +19348,7 @@
         <v>0</v>
       </c>
       <c r="R194" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S194" s="75" t="b">
         <v>0</v>
@@ -19392,7 +19392,7 @@
         <v>1873</v>
       </c>
       <c r="K195" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L195" s="64" t="b">
         <v>0</v>
@@ -19411,7 +19411,7 @@
         <v>0</v>
       </c>
       <c r="R195" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S195" s="75" t="b">
         <v>0</v>
@@ -19455,7 +19455,7 @@
         <v>1697</v>
       </c>
       <c r="K196" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L196" s="64" t="b">
         <v>0</v>
@@ -19474,7 +19474,7 @@
         <v>0</v>
       </c>
       <c r="R196" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S196" s="75" t="b">
         <v>0</v>
@@ -19518,7 +19518,7 @@
         <v>1782</v>
       </c>
       <c r="K197" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L197" s="64" t="b">
         <v>0</v>
@@ -19537,7 +19537,7 @@
         <v>0</v>
       </c>
       <c r="R197" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S197" s="75" t="b">
         <v>0</v>
@@ -19581,7 +19581,7 @@
         <v>1921</v>
       </c>
       <c r="K198" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L198" s="64" t="b">
         <v>0</v>
@@ -19600,7 +19600,7 @@
         <v>0</v>
       </c>
       <c r="R198" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S198" s="75" t="b">
         <v>0</v>
@@ -19644,7 +19644,7 @@
         <v>1795</v>
       </c>
       <c r="K199" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L199" s="64" t="b">
         <v>0</v>
@@ -19663,7 +19663,7 @@
         <v>0</v>
       </c>
       <c r="R199" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S199" s="75" t="b">
         <v>0</v>
@@ -19707,7 +19707,7 @@
         <v>1835</v>
       </c>
       <c r="K200" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L200" s="64" t="b">
         <v>0</v>
@@ -19726,7 +19726,7 @@
         <v>0</v>
       </c>
       <c r="R200" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S200" s="75" t="b">
         <v>0</v>
@@ -19770,7 +19770,7 @@
         <v>1794</v>
       </c>
       <c r="K201" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L201" s="64" t="b">
         <v>0</v>
@@ -19789,7 +19789,7 @@
         <v>0</v>
       </c>
       <c r="R201" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S201" s="75" t="b">
         <v>0</v>
@@ -19876,7 +19876,7 @@
         <v>1909</v>
       </c>
       <c r="K203" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L203" s="64" t="b">
         <v>0</v>
@@ -19895,7 +19895,7 @@
         <v>0</v>
       </c>
       <c r="R203" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S203" s="75" t="b">
         <v>0</v>
@@ -19937,7 +19937,7 @@
       </c>
       <c r="J204" s="18"/>
       <c r="K204" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L204" s="64" t="b">
         <v>0</v>
@@ -19956,7 +19956,7 @@
         <v>0</v>
       </c>
       <c r="R204" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S204" s="75" t="b">
         <v>0</v>
@@ -20000,7 +20000,7 @@
         <v>1785</v>
       </c>
       <c r="K205" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L205" s="64" t="b">
         <v>0</v>
@@ -20019,7 +20019,7 @@
         <v>0</v>
       </c>
       <c r="R205" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S205" s="75" t="b">
         <v>0</v>
@@ -20063,7 +20063,7 @@
         <v>1692</v>
       </c>
       <c r="K206" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L206" s="64" t="b">
         <v>0</v>
@@ -20082,7 +20082,7 @@
         <v>0</v>
       </c>
       <c r="R206" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S206" s="75" t="b">
         <v>0</v>
@@ -20126,7 +20126,7 @@
         <v>1790</v>
       </c>
       <c r="K207" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L207" s="64" t="b">
         <v>0</v>
@@ -20145,7 +20145,7 @@
         <v>0</v>
       </c>
       <c r="R207" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S207" s="75" t="b">
         <v>0</v>
@@ -20189,7 +20189,7 @@
         <v>1809</v>
       </c>
       <c r="K208" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L208" s="64" t="b">
         <v>0</v>
@@ -20208,7 +20208,7 @@
         <v>0</v>
       </c>
       <c r="R208" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S208" s="75" t="b">
         <v>0</v>
@@ -20252,7 +20252,7 @@
         <v>1742</v>
       </c>
       <c r="K209" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L209" s="64" t="b">
         <v>0</v>
@@ -20271,7 +20271,7 @@
         <v>0</v>
       </c>
       <c r="R209" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S209" s="75" t="b">
         <v>0</v>
@@ -20315,7 +20315,7 @@
         <v>1911</v>
       </c>
       <c r="K210" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L210" s="64" t="b">
         <v>0</v>
@@ -20334,7 +20334,7 @@
         <v>0</v>
       </c>
       <c r="R210" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S210" s="75" t="b">
         <v>0</v>
@@ -20378,7 +20378,7 @@
         <v>1898</v>
       </c>
       <c r="K211" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L211" s="64" t="b">
         <v>0</v>
@@ -20397,7 +20397,7 @@
         <v>0</v>
       </c>
       <c r="R211" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S211" s="75" t="b">
         <v>0</v>
@@ -20441,7 +20441,7 @@
         <v>1829</v>
       </c>
       <c r="K212" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L212" s="64" t="b">
         <v>0</v>
@@ -20460,7 +20460,7 @@
         <v>0</v>
       </c>
       <c r="R212" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S212" s="75" t="b">
         <v>0</v>
@@ -20504,7 +20504,7 @@
         <v>1786</v>
       </c>
       <c r="K213" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L213" s="64" t="b">
         <v>0</v>
@@ -20523,7 +20523,7 @@
         <v>0</v>
       </c>
       <c r="R213" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S213" s="75" t="b">
         <v>0</v>
@@ -20560,19 +20560,19 @@
       </c>
       <c r="J214" s="18"/>
       <c r="K214" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L214" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M214" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N214" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O214" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P214" s="55"/>
       <c r="Q214" s="74" t="b">
@@ -20623,7 +20623,7 @@
         <v>1773</v>
       </c>
       <c r="K215" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L215" s="64" t="b">
         <v>0</v>
@@ -20642,7 +20642,7 @@
         <v>0</v>
       </c>
       <c r="R215" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S215" s="75" t="b">
         <v>0</v>
@@ -20702,7 +20702,7 @@
       </c>
       <c r="P216" s="55"/>
       <c r="Q216" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R216" s="75" t="b">
         <v>0</v>
@@ -20749,7 +20749,7 @@
         <v>1744</v>
       </c>
       <c r="K217" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L217" s="64" t="b">
         <v>0</v>
@@ -20768,7 +20768,7 @@
         <v>0</v>
       </c>
       <c r="R217" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S217" s="75" t="b">
         <v>0</v>
@@ -20812,7 +20812,7 @@
         <v>1769</v>
       </c>
       <c r="K218" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L218" s="64" t="b">
         <v>0</v>
@@ -20831,7 +20831,7 @@
         <v>0</v>
       </c>
       <c r="R218" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S218" s="75" t="b">
         <v>0</v>
@@ -20873,7 +20873,7 @@
       </c>
       <c r="J219" s="18"/>
       <c r="K219" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L219" s="64" t="b">
         <v>0</v>
@@ -20892,7 +20892,7 @@
         <v>0</v>
       </c>
       <c r="R219" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S219" s="75" t="b">
         <v>0</v>
@@ -20936,7 +20936,7 @@
         <v>1887</v>
       </c>
       <c r="K220" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L220" s="64" t="b">
         <v>0</v>
@@ -20955,7 +20955,7 @@
         <v>0</v>
       </c>
       <c r="R220" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S220" s="75" t="b">
         <v>0</v>
@@ -20999,7 +20999,7 @@
         <v>1808</v>
       </c>
       <c r="K221" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L221" s="64" t="b">
         <v>0</v>
@@ -21018,7 +21018,7 @@
         <v>0</v>
       </c>
       <c r="R221" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S221" s="75" t="b">
         <v>0</v>
@@ -21062,7 +21062,7 @@
         <v>1834</v>
       </c>
       <c r="K222" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L222" s="64" t="b">
         <v>0</v>
@@ -21081,7 +21081,7 @@
         <v>0</v>
       </c>
       <c r="R222" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S222" s="75" t="b">
         <v>0</v>
@@ -21125,7 +21125,7 @@
         <v>1821</v>
       </c>
       <c r="K223" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L223" s="64" t="b">
         <v>0</v>
@@ -21144,7 +21144,7 @@
         <v>0</v>
       </c>
       <c r="R223" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S223" s="75" t="b">
         <v>0</v>
@@ -21188,7 +21188,7 @@
         <v>1871</v>
       </c>
       <c r="K224" s="66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L224" s="67" t="b">
         <v>0</v>
@@ -21207,7 +21207,7 @@
         <v>0</v>
       </c>
       <c r="R224" s="78" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S224" s="78" t="b">
         <v>0</v>
@@ -21251,7 +21251,7 @@
         <v>1882</v>
       </c>
       <c r="K225" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L225" s="64" t="b">
         <v>0</v>
@@ -21270,7 +21270,7 @@
         <v>0</v>
       </c>
       <c r="R225" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S225" s="75" t="b">
         <v>0</v>
@@ -21312,7 +21312,7 @@
       </c>
       <c r="J226" s="18"/>
       <c r="K226" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L226" s="64" t="b">
         <v>0</v>
@@ -21331,7 +21331,7 @@
         <v>0</v>
       </c>
       <c r="R226" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S226" s="75" t="b">
         <v>0</v>
@@ -21375,7 +21375,7 @@
         <v>1756</v>
       </c>
       <c r="K227" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L227" s="64" t="b">
         <v>0</v>
@@ -21394,7 +21394,7 @@
         <v>0</v>
       </c>
       <c r="R227" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S227" s="75" t="b">
         <v>0</v>
@@ -21438,7 +21438,7 @@
         <v>1747</v>
       </c>
       <c r="K228" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L228" s="64" t="b">
         <v>0</v>
@@ -21457,7 +21457,7 @@
         <v>0</v>
       </c>
       <c r="R228" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S228" s="75" t="b">
         <v>0</v>
@@ -21501,7 +21501,7 @@
         <v>1710</v>
       </c>
       <c r="K229" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L229" s="64" t="b">
         <v>0</v>
@@ -21520,7 +21520,7 @@
         <v>0</v>
       </c>
       <c r="R229" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S229" s="75" t="b">
         <v>0</v>
@@ -21564,7 +21564,7 @@
         <v>1819</v>
       </c>
       <c r="K230" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L230" s="64" t="b">
         <v>0</v>
@@ -21583,7 +21583,7 @@
         <v>0</v>
       </c>
       <c r="R230" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S230" s="75" t="b">
         <v>0</v>
@@ -21625,7 +21625,7 @@
       </c>
       <c r="J231" s="18"/>
       <c r="K231" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L231" s="64" t="b">
         <v>0</v>
@@ -21644,7 +21644,7 @@
         <v>0</v>
       </c>
       <c r="R231" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S231" s="75" t="b">
         <v>0</v>
@@ -21688,19 +21688,19 @@
         <v>1879</v>
       </c>
       <c r="K232" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L232" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M232" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N232" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O232" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P232" s="55"/>
       <c r="Q232" s="74" t="b">
@@ -21749,7 +21749,7 @@
       </c>
       <c r="J233" s="18"/>
       <c r="K233" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L233" s="64" t="b">
         <v>0</v>
@@ -21768,7 +21768,7 @@
         <v>0</v>
       </c>
       <c r="R233" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S233" s="75" t="b">
         <v>0</v>
@@ -21812,7 +21812,7 @@
         <v>1746</v>
       </c>
       <c r="K234" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L234" s="64" t="b">
         <v>0</v>
@@ -21831,7 +21831,7 @@
         <v>0</v>
       </c>
       <c r="R234" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S234" s="75" t="b">
         <v>0</v>
@@ -21875,7 +21875,7 @@
         <v>1868</v>
       </c>
       <c r="K235" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L235" s="64" t="b">
         <v>0</v>
@@ -21894,7 +21894,7 @@
         <v>0</v>
       </c>
       <c r="R235" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S235" s="75" t="b">
         <v>0</v>
@@ -21934,7 +21934,7 @@
       </c>
       <c r="J236" s="18"/>
       <c r="K236" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L236" s="64" t="b">
         <v>0</v>
@@ -21953,7 +21953,7 @@
         <v>0</v>
       </c>
       <c r="R236" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S236" s="75" t="b">
         <v>0</v>
@@ -21997,10 +21997,10 @@
         <v>1919</v>
       </c>
       <c r="K237" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L237" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M237" s="64" t="b">
         <v>0</v>
@@ -22019,7 +22019,7 @@
         <v>0</v>
       </c>
       <c r="S237" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T237" s="75" t="b">
         <v>0</v>
@@ -22060,7 +22060,7 @@
         <v>1703</v>
       </c>
       <c r="K238" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L238" s="64" t="b">
         <v>0</v>
@@ -22079,7 +22079,7 @@
         <v>0</v>
       </c>
       <c r="R238" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S238" s="75" t="b">
         <v>0</v>
@@ -22123,7 +22123,7 @@
         <v>1728</v>
       </c>
       <c r="K239" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L239" s="64" t="b">
         <v>0</v>
@@ -22142,7 +22142,7 @@
         <v>0</v>
       </c>
       <c r="R239" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S239" s="75" t="b">
         <v>0</v>
@@ -22227,7 +22227,7 @@
         <v>1718</v>
       </c>
       <c r="K241" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L241" s="64" t="b">
         <v>0</v>
@@ -22246,7 +22246,7 @@
         <v>0</v>
       </c>
       <c r="R241" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S241" s="75" t="b">
         <v>0</v>
@@ -22306,7 +22306,7 @@
       </c>
       <c r="P242" s="55"/>
       <c r="Q242" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R242" s="75" t="b">
         <v>0</v>
@@ -22351,7 +22351,7 @@
       </c>
       <c r="J243" s="18"/>
       <c r="K243" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L243" s="64" t="b">
         <v>0</v>
@@ -22370,7 +22370,7 @@
         <v>0</v>
       </c>
       <c r="R243" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S243" s="75" t="b">
         <v>0</v>
@@ -22455,7 +22455,7 @@
         <v>1792</v>
       </c>
       <c r="K245" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L245" s="64" t="b">
         <v>0</v>
@@ -22474,7 +22474,7 @@
         <v>0</v>
       </c>
       <c r="R245" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S245" s="75" t="b">
         <v>0</v>
@@ -22518,7 +22518,7 @@
         <v>1688</v>
       </c>
       <c r="K246" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L246" s="64" t="b">
         <v>0</v>
@@ -22537,7 +22537,7 @@
         <v>0</v>
       </c>
       <c r="R246" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S246" s="75" t="b">
         <v>0</v>
@@ -22581,7 +22581,7 @@
         <v>1698</v>
       </c>
       <c r="K247" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L247" s="64" t="b">
         <v>0</v>
@@ -22600,7 +22600,7 @@
         <v>0</v>
       </c>
       <c r="R247" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S247" s="75" t="b">
         <v>0</v>
@@ -22644,7 +22644,7 @@
         <v>1883</v>
       </c>
       <c r="K248" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L248" s="64" t="b">
         <v>0</v>
@@ -22663,7 +22663,7 @@
         <v>0</v>
       </c>
       <c r="R248" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S248" s="75" t="b">
         <v>0</v>
@@ -22707,7 +22707,7 @@
         <v>1826</v>
       </c>
       <c r="K249" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L249" s="64" t="b">
         <v>0</v>
@@ -22726,7 +22726,7 @@
         <v>0</v>
       </c>
       <c r="R249" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S249" s="75" t="b">
         <v>0</v>
@@ -22770,7 +22770,7 @@
         <v>1802</v>
       </c>
       <c r="K250" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L250" s="64" t="b">
         <v>0</v>
@@ -22789,7 +22789,7 @@
         <v>0</v>
       </c>
       <c r="R250" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S250" s="75" t="b">
         <v>0</v>
@@ -22831,7 +22831,7 @@
       </c>
       <c r="J251" s="18"/>
       <c r="K251" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L251" s="64" t="b">
         <v>0</v>
@@ -22850,7 +22850,7 @@
         <v>0</v>
       </c>
       <c r="R251" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S251" s="75" t="b">
         <v>0</v>
@@ -22894,7 +22894,7 @@
         <v>1706</v>
       </c>
       <c r="K252" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L252" s="64" t="b">
         <v>0</v>
@@ -22913,7 +22913,7 @@
         <v>0</v>
       </c>
       <c r="R252" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S252" s="75" t="b">
         <v>0</v>
@@ -22957,7 +22957,7 @@
         <v>1772</v>
       </c>
       <c r="K253" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L253" s="64" t="b">
         <v>0</v>
@@ -22976,7 +22976,7 @@
         <v>0</v>
       </c>
       <c r="R253" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S253" s="75" t="b">
         <v>0</v>
@@ -23020,7 +23020,7 @@
         <v>1828</v>
       </c>
       <c r="K254" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L254" s="64" t="b">
         <v>0</v>
@@ -23039,7 +23039,7 @@
         <v>0</v>
       </c>
       <c r="R254" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S254" s="75" t="b">
         <v>0</v>
@@ -23083,7 +23083,7 @@
         <v>1800</v>
       </c>
       <c r="K255" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L255" s="64" t="b">
         <v>0</v>
@@ -23102,7 +23102,7 @@
         <v>0</v>
       </c>
       <c r="R255" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S255" s="75" t="b">
         <v>0</v>
@@ -23146,7 +23146,7 @@
         <v>1752</v>
       </c>
       <c r="K256" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L256" s="64" t="b">
         <v>0</v>
@@ -23165,7 +23165,7 @@
         <v>0</v>
       </c>
       <c r="R256" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S256" s="75" t="b">
         <v>0</v>
@@ -23209,7 +23209,7 @@
         <v>1776</v>
       </c>
       <c r="K257" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L257" s="64" t="b">
         <v>0</v>
@@ -23228,7 +23228,7 @@
         <v>0</v>
       </c>
       <c r="R257" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S257" s="75" t="b">
         <v>0</v>
@@ -23270,7 +23270,7 @@
       </c>
       <c r="J258" s="18"/>
       <c r="K258" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L258" s="64" t="b">
         <v>0</v>
@@ -23289,7 +23289,7 @@
         <v>0</v>
       </c>
       <c r="R258" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S258" s="75" t="b">
         <v>0</v>
@@ -23333,7 +23333,7 @@
         <v>1770</v>
       </c>
       <c r="K259" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L259" s="64" t="b">
         <v>0</v>
@@ -23352,7 +23352,7 @@
         <v>0</v>
       </c>
       <c r="R259" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S259" s="75" t="b">
         <v>0</v>
@@ -23396,7 +23396,7 @@
         <v>1777</v>
       </c>
       <c r="K260" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L260" s="64" t="b">
         <v>0</v>
@@ -23415,7 +23415,7 @@
         <v>0</v>
       </c>
       <c r="R260" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S260" s="75" t="b">
         <v>0</v>
@@ -23457,7 +23457,7 @@
       </c>
       <c r="J261" s="18"/>
       <c r="K261" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L261" s="64" t="b">
         <v>0</v>
@@ -23476,7 +23476,7 @@
         <v>0</v>
       </c>
       <c r="R261" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S261" s="75" t="b">
         <v>0</v>
@@ -23520,19 +23520,19 @@
         <v>1771</v>
       </c>
       <c r="K262" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L262" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M262" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N262" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O262" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P262" s="55"/>
       <c r="Q262" s="74" t="b">
@@ -23583,19 +23583,19 @@
         <v>1908</v>
       </c>
       <c r="K263" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L263" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M263" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N263" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O263" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P263" s="55"/>
       <c r="Q263" s="74" t="b">
@@ -23646,7 +23646,7 @@
         <v>1715</v>
       </c>
       <c r="K264" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L264" s="64" t="b">
         <v>0</v>
@@ -23665,7 +23665,7 @@
         <v>0</v>
       </c>
       <c r="R264" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S264" s="75" t="b">
         <v>0</v>
@@ -23709,7 +23709,7 @@
         <v>1856</v>
       </c>
       <c r="K265" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L265" s="64" t="b">
         <v>0</v>
@@ -23728,7 +23728,7 @@
         <v>0</v>
       </c>
       <c r="R265" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S265" s="75" t="b">
         <v>0</v>
@@ -23772,7 +23772,7 @@
         <v>1783</v>
       </c>
       <c r="K266" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L266" s="64" t="b">
         <v>0</v>
@@ -23791,7 +23791,7 @@
         <v>0</v>
       </c>
       <c r="R266" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S266" s="75" t="b">
         <v>0</v>
@@ -23835,7 +23835,7 @@
         <v>1717</v>
       </c>
       <c r="K267" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L267" s="64" t="b">
         <v>0</v>
@@ -23854,7 +23854,7 @@
         <v>0</v>
       </c>
       <c r="R267" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S267" s="75" t="b">
         <v>0</v>
@@ -23898,7 +23898,7 @@
         <v>1731</v>
       </c>
       <c r="K268" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L268" s="64" t="b">
         <v>0</v>
@@ -23917,7 +23917,7 @@
         <v>0</v>
       </c>
       <c r="R268" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S268" s="75" t="b">
         <v>0</v>
@@ -23961,7 +23961,7 @@
         <v>1766</v>
       </c>
       <c r="K269" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L269" s="64" t="b">
         <v>0</v>
@@ -23980,7 +23980,7 @@
         <v>0</v>
       </c>
       <c r="R269" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S269" s="75" t="b">
         <v>0</v>
@@ -23992,7 +23992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A270" s="4" t="s">
         <v>10</v>
       </c>
@@ -24024,7 +24024,7 @@
         <v>1712</v>
       </c>
       <c r="K270" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L270" s="64" t="b">
         <v>0</v>
@@ -24043,7 +24043,7 @@
         <v>0</v>
       </c>
       <c r="R270" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S270" s="75" t="b">
         <v>0</v>
@@ -24087,19 +24087,19 @@
         <v>1796</v>
       </c>
       <c r="K271" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L271" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M271" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N271" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O271" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P271" s="55"/>
       <c r="Q271" s="74" t="b">
@@ -24150,19 +24150,19 @@
         <v>1758</v>
       </c>
       <c r="K272" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L272" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M272" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N272" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O272" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P272" s="55"/>
       <c r="Q272" s="74" t="b">
@@ -24213,7 +24213,7 @@
         <v>1780</v>
       </c>
       <c r="K273" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L273" s="64" t="b">
         <v>0</v>
@@ -24232,7 +24232,7 @@
         <v>0</v>
       </c>
       <c r="R273" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S273" s="75" t="b">
         <v>0</v>
@@ -24276,7 +24276,7 @@
         <v>1852</v>
       </c>
       <c r="K274" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L274" s="64" t="b">
         <v>0</v>
@@ -24295,7 +24295,7 @@
         <v>0</v>
       </c>
       <c r="R274" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S274" s="75" t="b">
         <v>0</v>
@@ -24307,7 +24307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:21" s="4" customFormat="1" ht="189" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:21" s="4" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A275" s="4" t="s">
         <v>12</v>
       </c>
@@ -24337,19 +24337,19 @@
       </c>
       <c r="J275" s="18"/>
       <c r="K275" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L275" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M275" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N275" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O275" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P275" s="55"/>
       <c r="Q275" s="74" t="b">
@@ -24400,7 +24400,7 @@
         <v>1733</v>
       </c>
       <c r="K276" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L276" s="64" t="b">
         <v>0</v>
@@ -24419,7 +24419,7 @@
         <v>0</v>
       </c>
       <c r="R276" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S276" s="75" t="b">
         <v>0</v>
@@ -24463,19 +24463,19 @@
         <v>1793</v>
       </c>
       <c r="K277" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L277" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M277" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N277" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O277" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P277" s="55"/>
       <c r="Q277" s="74" t="b">
@@ -24494,7 +24494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:21" s="4" customFormat="1" ht="223" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:21" s="4" customFormat="1" ht="240" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A278" s="4" t="s">
         <v>15</v>
       </c>
@@ -24526,7 +24526,7 @@
         <v>1922</v>
       </c>
       <c r="K278" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L278" s="64" t="b">
         <v>0</v>
@@ -24545,7 +24545,7 @@
         <v>0</v>
       </c>
       <c r="R278" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S278" s="75" t="b">
         <v>0</v>
@@ -24589,7 +24589,7 @@
         <v>1700</v>
       </c>
       <c r="K279" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L279" s="64" t="b">
         <v>0</v>
@@ -24608,7 +24608,7 @@
         <v>0</v>
       </c>
       <c r="R279" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S279" s="75" t="b">
         <v>0</v>
@@ -24652,7 +24652,7 @@
         <v>1755</v>
       </c>
       <c r="K280" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L280" s="64" t="b">
         <v>0</v>
@@ -24671,7 +24671,7 @@
         <v>0</v>
       </c>
       <c r="R280" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S280" s="75" t="b">
         <v>0</v>
@@ -24715,19 +24715,19 @@
         <v>1841</v>
       </c>
       <c r="K281" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L281" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M281" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N281" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O281" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P281" s="55"/>
       <c r="Q281" s="74" t="b">
@@ -24794,7 +24794,7 @@
       </c>
       <c r="P282" s="55"/>
       <c r="Q282" s="74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R282" s="75" t="b">
         <v>0</v>
@@ -24841,7 +24841,7 @@
         <v>1813</v>
       </c>
       <c r="K283" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L283" s="64" t="b">
         <v>0</v>
@@ -24860,7 +24860,7 @@
         <v>0</v>
       </c>
       <c r="R283" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S283" s="75" t="b">
         <v>0</v>
@@ -24902,7 +24902,7 @@
       </c>
       <c r="J284" s="18"/>
       <c r="K284" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L284" s="64" t="b">
         <v>0</v>
@@ -24921,7 +24921,7 @@
         <v>0</v>
       </c>
       <c r="R284" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S284" s="75" t="b">
         <v>0</v>
@@ -24965,19 +24965,19 @@
         <v>1805</v>
       </c>
       <c r="K285" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L285" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M285" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N285" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O285" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P285" s="55"/>
       <c r="Q285" s="74" t="b">
@@ -25028,7 +25028,7 @@
         <v>1880</v>
       </c>
       <c r="K286" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L286" s="64" t="b">
         <v>0</v>
@@ -25047,7 +25047,7 @@
         <v>0</v>
       </c>
       <c r="R286" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S286" s="75" t="b">
         <v>0</v>
@@ -25091,7 +25091,7 @@
         <v>1709</v>
       </c>
       <c r="K287" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L287" s="64" t="b">
         <v>0</v>
@@ -25110,7 +25110,7 @@
         <v>0</v>
       </c>
       <c r="R287" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S287" s="75" t="b">
         <v>0</v>
@@ -25154,19 +25154,19 @@
         <v>1915</v>
       </c>
       <c r="K288" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L288" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M288" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N288" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O288" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P288" s="55"/>
       <c r="Q288" s="74" t="b">
@@ -25217,7 +25217,7 @@
         <v>1730</v>
       </c>
       <c r="K289" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L289" s="64" t="b">
         <v>0</v>
@@ -25236,7 +25236,7 @@
         <v>0</v>
       </c>
       <c r="R289" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S289" s="75" t="b">
         <v>0</v>
@@ -25280,7 +25280,7 @@
         <v>1848</v>
       </c>
       <c r="K290" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L290" s="64" t="b">
         <v>0</v>
@@ -25299,7 +25299,7 @@
         <v>0</v>
       </c>
       <c r="R290" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S290" s="75" t="b">
         <v>0</v>
@@ -25343,7 +25343,7 @@
         <v>1918</v>
       </c>
       <c r="K291" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L291" s="64" t="b">
         <v>0</v>
@@ -25362,7 +25362,7 @@
         <v>0</v>
       </c>
       <c r="R291" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S291" s="75" t="b">
         <v>0</v>
@@ -25402,7 +25402,7 @@
       </c>
       <c r="J292" s="18"/>
       <c r="K292" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L292" s="64" t="b">
         <v>0</v>
@@ -25421,7 +25421,7 @@
         <v>0</v>
       </c>
       <c r="R292" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S292" s="75" t="b">
         <v>0</v>
@@ -25465,7 +25465,7 @@
         <v>1714</v>
       </c>
       <c r="K293" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L293" s="64" t="b">
         <v>0</v>
@@ -25484,7 +25484,7 @@
         <v>0</v>
       </c>
       <c r="R293" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S293" s="75" t="b">
         <v>0</v>
@@ -25528,7 +25528,7 @@
         <v>1926</v>
       </c>
       <c r="K294" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L294" s="64" t="b">
         <v>0</v>
@@ -25547,7 +25547,7 @@
         <v>0</v>
       </c>
       <c r="R294" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S294" s="75" t="b">
         <v>0</v>
@@ -25591,19 +25591,19 @@
         <v>1801</v>
       </c>
       <c r="K295" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L295" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M295" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N295" s="64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O295" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P295" s="55"/>
       <c r="Q295" s="74" t="b">
@@ -25654,7 +25654,7 @@
         <v>1822</v>
       </c>
       <c r="K296" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L296" s="64" t="b">
         <v>0</v>
@@ -25673,7 +25673,7 @@
         <v>0</v>
       </c>
       <c r="R296" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S296" s="75" t="b">
         <v>0</v>
@@ -25717,7 +25717,7 @@
         <v>1789</v>
       </c>
       <c r="K297" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L297" s="64" t="b">
         <v>0</v>
@@ -25736,7 +25736,7 @@
         <v>0</v>
       </c>
       <c r="R297" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S297" s="75" t="b">
         <v>0</v>
@@ -25780,7 +25780,7 @@
         <v>1779</v>
       </c>
       <c r="K298" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L298" s="64" t="b">
         <v>0</v>
@@ -25799,7 +25799,7 @@
         <v>0</v>
       </c>
       <c r="R298" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S298" s="75" t="b">
         <v>0</v>
@@ -25843,7 +25843,7 @@
         <v>1924</v>
       </c>
       <c r="K299" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L299" s="64" t="b">
         <v>0</v>
@@ -25862,7 +25862,7 @@
         <v>0</v>
       </c>
       <c r="R299" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S299" s="75" t="b">
         <v>0</v>
@@ -25904,7 +25904,7 @@
       </c>
       <c r="J300" s="18"/>
       <c r="K300" s="63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L300" s="64" t="b">
         <v>0</v>
@@ -25923,7 +25923,7 @@
         <v>0</v>
       </c>
       <c r="R300" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S300" s="75" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
add summary excel for second screening and preliminary citation searching/results excel sheets
</commit_message>
<xml_diff>
--- a/lit_review_results/2-screening_phase/second_screening_reviewer_A.xlsx
+++ b/lit_review_results/2-screening_phase/second_screening_reviewer_A.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wolfrieder/PycharmProjects/sok_artifacts/lit_review_results/2-screening_phase/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{311212DC-5D48-C641-84CB-7A784534935D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20FE2271-ED05-4045-8703-0F8CDDB7BA4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7740" yWindow="-28240" windowWidth="51080" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60" yWindow="940" windowWidth="35880" windowHeight="21320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7919,7 +7919,7 @@
         <v>0</v>
       </c>
       <c r="R11" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" s="75" t="b">
         <v>0</v>
@@ -8594,23 +8594,23 @@
         <v>1</v>
       </c>
       <c r="L22" s="64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22" s="64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N22" s="64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O22" s="65" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P22" s="55"/>
       <c r="Q22" s="74" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R22" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S22" s="75" t="b">
         <v>0</v>
@@ -10561,7 +10561,7 @@
         <v>0</v>
       </c>
       <c r="R53" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S53" s="75" t="b">
         <v>0</v>
@@ -11124,7 +11124,7 @@
         <v>0</v>
       </c>
       <c r="R62" s="75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S62" s="75" t="b">
         <v>0</v>
@@ -12227,7 +12227,7 @@
         <v>1</v>
       </c>
       <c r="O80" s="65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P80" s="55"/>
       <c r="Q80" s="74" t="b">

</xml_diff>